<commit_message>
auto: actualizar indicadores adelantados 2026-06-29
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
+++ b/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PARA LA WEB\CONSUMO ELECTRICO\INDICADORES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PARA LA WEB - ABRIL\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11430"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
   </bookViews>
   <sheets>
     <sheet name="Índice" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="38">
   <si>
     <t>DOMÉSTICO</t>
   </si>
@@ -1099,7 +1099,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="B1:W167"/>
+  <dimension ref="B1:W168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -4533,25 +4533,25 @@
         <v>33</v>
       </c>
       <c r="C132" s="10">
-        <v>131.03815916195799</v>
+        <v>130.79537920294501</v>
       </c>
       <c r="D132" s="10">
-        <v>130.657387336352</v>
+        <v>131.77926673946001</v>
       </c>
       <c r="E132" s="10">
-        <v>119.698827458664</v>
+        <v>122.510722209119</v>
       </c>
       <c r="F132" s="10">
-        <v>170.85148041978999</v>
+        <v>175.89263798508301</v>
       </c>
       <c r="G132" s="10">
-        <v>109.71068458080001</v>
+        <v>115.221935986085</v>
       </c>
       <c r="H132" s="10">
-        <v>158.47578257735699</v>
+        <v>159.40834080794701</v>
       </c>
       <c r="I132" s="10">
-        <v>130.49034308661899</v>
+        <v>131.85001427717</v>
       </c>
     </row>
     <row r="133" spans="2:9">
@@ -4562,7 +4562,7 @@
         <v>133.81745310174699</v>
       </c>
       <c r="D133" s="12">
-        <v>130.32145092270599</v>
+        <v>130.33319574657801</v>
       </c>
       <c r="E133" s="12">
         <v>117.55876343064899</v>
@@ -4574,10 +4574,10 @@
         <v>115.76923599584499</v>
       </c>
       <c r="H133" s="12">
-        <v>152.95335954972199</v>
+        <v>153.05492493059</v>
       </c>
       <c r="I133" s="12">
-        <v>131.280694947304</v>
+        <v>131.28751996418501</v>
       </c>
     </row>
     <row r="134" spans="2:9">
@@ -4588,7 +4588,7 @@
         <v>130.45201169262</v>
       </c>
       <c r="D134" s="12">
-        <v>130.906667639245</v>
+        <v>130.91666595341499</v>
       </c>
       <c r="E134" s="12">
         <v>117.182631524885</v>
@@ -4600,94 +4600,111 @@
         <v>100.515598973637</v>
       </c>
       <c r="H134" s="12">
-        <v>153.68545185153701</v>
+        <v>153.79914306051501</v>
       </c>
       <c r="I134" s="12">
-        <v>129.26992927640501</v>
+        <v>129.276682334128</v>
       </c>
     </row>
     <row r="135" spans="2:9">
-      <c r="B135" s="33" t="s">
+      <c r="B135" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C135" s="16">
+      <c r="C135" s="12">
         <v>128.84501269150601</v>
       </c>
-      <c r="D135" s="16">
-        <v>130.74404344710601</v>
-      </c>
-      <c r="E135" s="16">
-        <v>124.355087420457</v>
-      </c>
-      <c r="F135" s="16">
+      <c r="D135" s="12">
+        <v>130.76976107479501</v>
+      </c>
+      <c r="E135" s="12">
+        <v>124.35357664608399</v>
+      </c>
+      <c r="F135" s="12">
         <v>168.02622962471301</v>
       </c>
-      <c r="G135" s="16">
+      <c r="G135" s="12">
         <v>112.84721877291901</v>
       </c>
-      <c r="H135" s="16">
-        <v>168.78853633081201</v>
-      </c>
-      <c r="I135" s="16">
-        <v>130.920405036147</v>
-      </c>
-    </row>
-    <row r="136" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B136" s="29" t="s">
+      <c r="H135" s="12">
+        <v>168.896268759755</v>
+      </c>
+      <c r="I135" s="12">
+        <v>130.931102875064</v>
+      </c>
+    </row>
+    <row r="136" spans="2:9">
+      <c r="B136" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" s="16">
+        <v>130.06703932590801</v>
+      </c>
+      <c r="D136" s="16">
+        <v>135.09744418304999</v>
+      </c>
+      <c r="E136" s="16">
+        <v>130.94791723485801</v>
+      </c>
+      <c r="F136" s="16">
+        <v>191.016110680964</v>
+      </c>
+      <c r="G136" s="16">
+        <v>131.75569020193799</v>
+      </c>
+      <c r="H136" s="16">
+        <v>161.88302648092599</v>
+      </c>
+      <c r="I136" s="16">
+        <v>135.904751935305</v>
+      </c>
+    </row>
+    <row r="137" spans="2:9" ht="14.25" customHeight="1">
+      <c r="B137" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C136" s="30"/>
-      <c r="D136" s="30"/>
-      <c r="E136" s="30"/>
-      <c r="F136" s="30"/>
-      <c r="G136" s="30"/>
-      <c r="H136" s="30"/>
-      <c r="I136" s="30"/>
-    </row>
-    <row r="137" spans="2:9" ht="34.5" customHeight="1">
-      <c r="B137" s="35" t="s">
+      <c r="C137" s="30"/>
+      <c r="D137" s="30"/>
+      <c r="E137" s="30"/>
+      <c r="F137" s="30"/>
+      <c r="G137" s="30"/>
+      <c r="H137" s="30"/>
+      <c r="I137" s="30"/>
+    </row>
+    <row r="138" spans="2:9" ht="34.5" customHeight="1">
+      <c r="B138" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C137" s="35"/>
-      <c r="D137" s="35"/>
-      <c r="E137" s="35"/>
-      <c r="F137" s="35"/>
-      <c r="G137" s="35"/>
-      <c r="H137" s="35"/>
-      <c r="I137" s="35"/>
-    </row>
-    <row r="138" spans="2:9">
-      <c r="B138" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C138" s="32"/>
-      <c r="D138" s="32"/>
-      <c r="E138" s="32"/>
-      <c r="F138" s="32"/>
-      <c r="G138" s="32"/>
-      <c r="H138" s="32"/>
-      <c r="I138" s="32"/>
+      <c r="C138" s="35"/>
+      <c r="D138" s="35"/>
+      <c r="E138" s="35"/>
+      <c r="F138" s="35"/>
+      <c r="G138" s="35"/>
+      <c r="H138" s="35"/>
+      <c r="I138" s="35"/>
     </row>
     <row r="139" spans="2:9">
       <c r="B139" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C139" s="32"/>
+      <c r="D139" s="32"/>
+      <c r="E139" s="32"/>
+      <c r="F139" s="32"/>
+      <c r="G139" s="32"/>
+      <c r="H139" s="32"/>
+      <c r="I139" s="32"/>
+    </row>
+    <row r="140" spans="2:9">
+      <c r="B140" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C139" s="30"/>
-      <c r="D139" s="30"/>
-      <c r="E139" s="30"/>
-      <c r="F139" s="30"/>
-      <c r="G139" s="30"/>
-      <c r="H139" s="30"/>
-      <c r="I139" s="30"/>
-    </row>
-    <row r="141" spans="2:9">
-      <c r="C141" s="17"/>
-      <c r="D141" s="17"/>
-      <c r="E141" s="17"/>
-      <c r="F141" s="17"/>
-      <c r="G141" s="17"/>
-      <c r="H141" s="17"/>
-      <c r="I141" s="17"/>
+      <c r="C140" s="30"/>
+      <c r="D140" s="30"/>
+      <c r="E140" s="30"/>
+      <c r="F140" s="30"/>
+      <c r="G140" s="30"/>
+      <c r="H140" s="30"/>
+      <c r="I140" s="30"/>
     </row>
     <row r="142" spans="2:9">
       <c r="C142" s="17"/>
@@ -4843,13 +4860,13 @@
       <c r="I158" s="17"/>
     </row>
     <row r="159" spans="3:9">
-      <c r="C159" s="18"/>
-      <c r="D159" s="18"/>
-      <c r="E159" s="18"/>
-      <c r="F159" s="18"/>
-      <c r="G159" s="18"/>
-      <c r="H159" s="18"/>
-      <c r="I159" s="18"/>
+      <c r="C159" s="17"/>
+      <c r="D159" s="17"/>
+      <c r="E159" s="17"/>
+      <c r="F159" s="17"/>
+      <c r="G159" s="17"/>
+      <c r="H159" s="17"/>
+      <c r="I159" s="17"/>
     </row>
     <row r="160" spans="3:9">
       <c r="C160" s="18"/>
@@ -4923,10 +4940,19 @@
       <c r="H167" s="18"/>
       <c r="I167" s="18"/>
     </row>
+    <row r="168" spans="3:9">
+      <c r="C168" s="18"/>
+      <c r="D168" s="18"/>
+      <c r="E168" s="18"/>
+      <c r="F168" s="18"/>
+      <c r="G168" s="18"/>
+      <c r="H168" s="18"/>
+      <c r="I168" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B137:I137"/>
+    <mergeCell ref="B138:I138"/>
     <mergeCell ref="B3:G3"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
@@ -4939,7 +4965,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja3"/>
-  <dimension ref="B1:K147"/>
+  <dimension ref="B1:K148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -7801,25 +7827,25 @@
         <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>1.35472311620472</v>
+        <v>4.6754931053025501</v>
       </c>
       <c r="D118" s="10">
-        <v>1.03127330483505</v>
+        <v>3.6364812084440001</v>
       </c>
       <c r="E118" s="10">
-        <v>-1.8971807729040899</v>
+        <v>-2.9324445375819299</v>
       </c>
       <c r="F118" s="10">
-        <v>15.788420066365999</v>
+        <v>16.038477753051101</v>
       </c>
       <c r="G118" s="10">
-        <v>-0.91298897139768098</v>
+        <v>1.8537277247402799</v>
       </c>
       <c r="H118" s="10">
-        <v>5.6650459659394699</v>
+        <v>5.9368459809194301</v>
       </c>
       <c r="I118" s="10">
-        <v>1.73046083411479</v>
+        <v>3.7909082765206801</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
@@ -7832,7 +7858,7 @@
         <v>7.3000843336288801</v>
       </c>
       <c r="D119" s="12">
-        <v>0.32910754787136598</v>
+        <v>0.33814940313814401</v>
       </c>
       <c r="E119" s="12">
         <v>-8.9783131613286002</v>
@@ -7844,10 +7870,10 @@
         <v>5.1591213604943702</v>
       </c>
       <c r="H119" s="12">
-        <v>-10.7782993246442</v>
+        <v>-10.719053577852801</v>
       </c>
       <c r="I119" s="12">
-        <v>0.44999697082788198</v>
+        <v>0.45521916229560599</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
@@ -7860,7 +7886,7 @@
         <v>-2.5149495309616499</v>
       </c>
       <c r="D120" s="12">
-        <v>0.44905632372516102</v>
+        <v>0.44767582310429899</v>
       </c>
       <c r="E120" s="12">
         <v>-0.31995224752927598</v>
@@ -7872,106 +7898,125 @@
         <v>-13.175898494099799</v>
       </c>
       <c r="H120" s="12">
-        <v>0.47863760820314699</v>
+        <v>0.48624252389308797</v>
       </c>
       <c r="I120" s="12">
-        <v>-1.5316537375935599</v>
+        <v>-1.5316289245204699</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
     </row>
     <row r="121" spans="2:11">
-      <c r="B121" s="33" t="s">
+      <c r="B121" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C121" s="16">
+      <c r="C121" s="12">
         <v>-1.23186985027123</v>
       </c>
-      <c r="D121" s="16">
-        <v>-0.12422911305523</v>
-      </c>
-      <c r="E121" s="16">
-        <v>6.1207499799561997</v>
-      </c>
-      <c r="F121" s="16">
+      <c r="D121" s="12">
+        <v>-0.112212511332987</v>
+      </c>
+      <c r="E121" s="12">
+        <v>6.1194607322641001</v>
+      </c>
+      <c r="F121" s="12">
         <v>-3.12210605626229</v>
       </c>
-      <c r="G121" s="16">
+      <c r="G121" s="12">
         <v>12.268364239182899</v>
       </c>
-      <c r="H121" s="16">
-        <v>9.8272701139364305</v>
-      </c>
-      <c r="I121" s="16">
-        <v>1.27676697046282</v>
+      <c r="H121" s="12">
+        <v>9.8161312207695897</v>
+      </c>
+      <c r="I121" s="12">
+        <v>1.2797517008208401</v>
       </c>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
     </row>
-    <row r="122" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B122" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C122" s="30"/>
-      <c r="D122" s="30"/>
-      <c r="E122" s="30"/>
-      <c r="F122" s="30"/>
-      <c r="G122" s="30"/>
-      <c r="H122" s="30"/>
-      <c r="I122" s="30"/>
+    <row r="122" spans="2:11">
+      <c r="B122" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C122" s="16">
+        <v>0.94844698205578404</v>
+      </c>
+      <c r="D122" s="16">
+        <v>3.3093913093407399</v>
+      </c>
+      <c r="E122" s="16">
+        <v>5.3028957965092403</v>
+      </c>
+      <c r="F122" s="16">
+        <v>13.682316807083801</v>
+      </c>
+      <c r="G122" s="16">
+        <v>16.755815193875701</v>
+      </c>
+      <c r="H122" s="16">
+        <v>-4.1523962194836797</v>
+      </c>
+      <c r="I122" s="16">
+        <v>3.7986765184335298</v>
+      </c>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
     </row>
-    <row r="123" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B123" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C123" s="35"/>
-      <c r="D123" s="35"/>
-      <c r="E123" s="35"/>
-      <c r="F123" s="35"/>
-      <c r="G123" s="35"/>
-      <c r="H123" s="35"/>
-      <c r="I123" s="35"/>
+    <row r="123" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B123" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C123" s="30"/>
+      <c r="D123" s="30"/>
+      <c r="E123" s="30"/>
+      <c r="F123" s="30"/>
+      <c r="G123" s="30"/>
+      <c r="H123" s="30"/>
+      <c r="I123" s="30"/>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
     </row>
-    <row r="124" spans="2:11">
-      <c r="B124" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C124" s="32"/>
-      <c r="D124" s="32"/>
-      <c r="E124" s="32"/>
-      <c r="F124" s="32"/>
-      <c r="G124" s="32"/>
-      <c r="H124" s="32"/>
-      <c r="I124" s="32"/>
+    <row r="124" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B124" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C124" s="35"/>
+      <c r="D124" s="35"/>
+      <c r="E124" s="35"/>
+      <c r="F124" s="35"/>
+      <c r="G124" s="35"/>
+      <c r="H124" s="35"/>
+      <c r="I124" s="35"/>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
     </row>
     <row r="125" spans="2:11">
       <c r="B125" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C125" s="30"/>
-      <c r="D125" s="30"/>
-      <c r="E125" s="30"/>
-      <c r="F125" s="30"/>
-      <c r="G125" s="30"/>
-      <c r="H125" s="30"/>
-      <c r="I125" s="30"/>
+        <v>24</v>
+      </c>
+      <c r="C125" s="32"/>
+      <c r="D125" s="32"/>
+      <c r="E125" s="32"/>
+      <c r="F125" s="32"/>
+      <c r="G125" s="32"/>
+      <c r="H125" s="32"/>
+      <c r="I125" s="32"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
     </row>
     <row r="126" spans="2:11">
-      <c r="C126" s="19"/>
-      <c r="D126" s="19"/>
-      <c r="E126" s="19"/>
-      <c r="F126" s="19"/>
-      <c r="G126" s="19"/>
-      <c r="H126" s="19"/>
-      <c r="I126" s="19"/>
+      <c r="B126" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C126" s="30"/>
+      <c r="D126" s="30"/>
+      <c r="E126" s="30"/>
+      <c r="F126" s="30"/>
+      <c r="G126" s="30"/>
+      <c r="H126" s="30"/>
+      <c r="I126" s="30"/>
+      <c r="J126" s="1"/>
+      <c r="K126" s="1"/>
     </row>
     <row r="127" spans="2:11">
       <c r="C127" s="19"/>
@@ -8010,13 +8055,13 @@
       <c r="I130" s="19"/>
     </row>
     <row r="131" spans="3:9">
-      <c r="C131" s="17"/>
-      <c r="D131" s="17"/>
-      <c r="E131" s="17"/>
-      <c r="F131" s="17"/>
-      <c r="G131" s="17"/>
-      <c r="H131" s="17"/>
-      <c r="I131" s="17"/>
+      <c r="C131" s="19"/>
+      <c r="D131" s="19"/>
+      <c r="E131" s="19"/>
+      <c r="F131" s="19"/>
+      <c r="G131" s="19"/>
+      <c r="H131" s="19"/>
+      <c r="I131" s="19"/>
     </row>
     <row r="132" spans="3:9">
       <c r="C132" s="17"/>
@@ -8162,10 +8207,19 @@
       <c r="H147" s="17"/>
       <c r="I147" s="17"/>
     </row>
+    <row r="148" spans="3:9">
+      <c r="C148" s="17"/>
+      <c r="D148" s="17"/>
+      <c r="E148" s="17"/>
+      <c r="F148" s="17"/>
+      <c r="G148" s="17"/>
+      <c r="H148" s="17"/>
+      <c r="I148" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B123:I123"/>
+    <mergeCell ref="B124:I124"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8177,7 +8231,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="B1:K156"/>
+  <dimension ref="B1:K157"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -11039,25 +11093,25 @@
         <v>37</v>
       </c>
       <c r="C118" s="10">
-        <v>1.35472311620472</v>
+        <v>4.6754931053025501</v>
       </c>
       <c r="D118" s="10">
-        <v>1.03127330483505</v>
+        <v>3.6364812084440001</v>
       </c>
       <c r="E118" s="10">
-        <v>-1.8971807729040899</v>
+        <v>-2.9324445375819299</v>
       </c>
       <c r="F118" s="10">
-        <v>15.788420066365999</v>
+        <v>16.038477753051101</v>
       </c>
       <c r="G118" s="10">
-        <v>-0.91298897139768098</v>
+        <v>1.8537277247402799</v>
       </c>
       <c r="H118" s="10">
-        <v>5.6650459659394699</v>
+        <v>5.9368459809194301</v>
       </c>
       <c r="I118" s="10">
-        <v>1.73046083411479</v>
+        <v>3.7909082765206801</v>
       </c>
       <c r="K118" s="1"/>
     </row>
@@ -11069,7 +11123,7 @@
         <v>3.72865534857034</v>
       </c>
       <c r="D119" s="12">
-        <v>2.7568523330344901</v>
+        <v>2.7661129814063901</v>
       </c>
       <c r="E119" s="12">
         <v>-2.5515743658463301</v>
@@ -11081,10 +11135,10 @@
         <v>6.0160708382844801</v>
       </c>
       <c r="H119" s="12">
-        <v>-5.3237302845463699</v>
+        <v>-5.2608625487796203</v>
       </c>
       <c r="I119" s="12">
-        <v>2.9133532378905</v>
+        <v>2.9187034942509</v>
       </c>
       <c r="K119" s="1"/>
     </row>
@@ -11096,7 +11150,7 @@
         <v>-1.0685583386863899</v>
       </c>
       <c r="D120" s="12">
-        <v>-0.36899580473565002</v>
+        <v>-0.36138624519996798</v>
       </c>
       <c r="E120" s="12">
         <v>-6.3351241779361596</v>
@@ -11108,100 +11162,118 @@
         <v>-6.4747464267629802</v>
       </c>
       <c r="H120" s="12">
-        <v>4.8365230382085196</v>
+        <v>4.9140774905373803</v>
       </c>
       <c r="I120" s="12">
-        <v>-0.827002129429522</v>
+        <v>-0.82182133461548001</v>
       </c>
       <c r="K120" s="1"/>
     </row>
     <row r="121" spans="2:11">
-      <c r="B121" s="33" t="s">
+      <c r="B121" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C121" s="16">
+      <c r="C121" s="12">
         <v>1.45931237591159</v>
       </c>
-      <c r="D121" s="16">
-        <v>0.76258732698875098</v>
-      </c>
-      <c r="E121" s="16">
-        <v>3.37456534505962</v>
-      </c>
-      <c r="F121" s="16">
+      <c r="D121" s="12">
+        <v>0.78240753934795104</v>
+      </c>
+      <c r="E121" s="12">
+        <v>3.3733094604205101</v>
+      </c>
+      <c r="F121" s="12">
         <v>19.799265689296799</v>
       </c>
-      <c r="G121" s="16">
+      <c r="G121" s="12">
         <v>-2.2889039419712902</v>
       </c>
-      <c r="H121" s="16">
-        <v>19.042264260389601</v>
-      </c>
-      <c r="I121" s="16">
-        <v>3.1683284232916198</v>
+      <c r="H121" s="12">
+        <v>19.118245204086499</v>
+      </c>
+      <c r="I121" s="12">
+        <v>3.1767585695207501</v>
       </c>
       <c r="K121" s="1"/>
     </row>
-    <row r="122" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B122" s="29" t="s">
+    <row r="122" spans="2:11">
+      <c r="B122" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C122" s="16">
+        <v>16.1802925760467</v>
+      </c>
+      <c r="D122" s="16">
+        <v>11.9746416696604</v>
+      </c>
+      <c r="E122" s="16">
+        <v>-5.6614115014834798</v>
+      </c>
+      <c r="F122" s="16">
+        <v>16.714827162760098</v>
+      </c>
+      <c r="G122" s="16">
+        <v>9.49079036829648</v>
+      </c>
+      <c r="H122" s="16">
+        <v>6.5290642010867197</v>
+      </c>
+      <c r="I122" s="16">
+        <v>10.200452758813</v>
+      </c>
+      <c r="K122" s="1"/>
+    </row>
+    <row r="123" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B123" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C122" s="30"/>
-      <c r="D122" s="30"/>
-      <c r="E122" s="30"/>
-      <c r="F122" s="30"/>
-      <c r="G122" s="30"/>
-      <c r="H122" s="30"/>
-      <c r="I122" s="30"/>
-      <c r="K122" s="1"/>
-    </row>
-    <row r="123" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B123" s="35" t="s">
+      <c r="C123" s="30"/>
+      <c r="D123" s="30"/>
+      <c r="E123" s="30"/>
+      <c r="F123" s="30"/>
+      <c r="G123" s="30"/>
+      <c r="H123" s="30"/>
+      <c r="I123" s="30"/>
+      <c r="K123" s="1"/>
+    </row>
+    <row r="124" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B124" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C123" s="35"/>
-      <c r="D123" s="35"/>
-      <c r="E123" s="35"/>
-      <c r="F123" s="35"/>
-      <c r="G123" s="35"/>
-      <c r="H123" s="35"/>
-      <c r="I123" s="35"/>
-      <c r="K123" s="1"/>
-    </row>
-    <row r="124" spans="2:11">
-      <c r="B124" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C124" s="32"/>
-      <c r="D124" s="32"/>
-      <c r="E124" s="32"/>
-      <c r="F124" s="32"/>
-      <c r="G124" s="32"/>
-      <c r="H124" s="32"/>
-      <c r="I124" s="32"/>
+      <c r="C124" s="35"/>
+      <c r="D124" s="35"/>
+      <c r="E124" s="35"/>
+      <c r="F124" s="35"/>
+      <c r="G124" s="35"/>
+      <c r="H124" s="35"/>
+      <c r="I124" s="35"/>
       <c r="K124" s="1"/>
     </row>
     <row r="125" spans="2:11">
       <c r="B125" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C125" s="32"/>
+      <c r="D125" s="32"/>
+      <c r="E125" s="32"/>
+      <c r="F125" s="32"/>
+      <c r="G125" s="32"/>
+      <c r="H125" s="32"/>
+      <c r="I125" s="32"/>
+      <c r="K125" s="1"/>
+    </row>
+    <row r="126" spans="2:11">
+      <c r="B126" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C125" s="30"/>
-      <c r="D125" s="30"/>
-      <c r="E125" s="30"/>
-      <c r="F125" s="30"/>
-      <c r="G125" s="30"/>
-      <c r="H125" s="30"/>
-      <c r="I125" s="30"/>
-      <c r="K125" s="1"/>
-    </row>
-    <row r="130" spans="3:9">
-      <c r="C130" s="17"/>
-      <c r="D130" s="17"/>
-      <c r="E130" s="17"/>
-      <c r="F130" s="17"/>
-      <c r="G130" s="17"/>
-      <c r="H130" s="17"/>
-      <c r="I130" s="17"/>
+      <c r="C126" s="30"/>
+      <c r="D126" s="30"/>
+      <c r="E126" s="30"/>
+      <c r="F126" s="30"/>
+      <c r="G126" s="30"/>
+      <c r="H126" s="30"/>
+      <c r="I126" s="30"/>
+      <c r="K126" s="1"/>
     </row>
     <row r="131" spans="3:9">
       <c r="C131" s="17"/>
@@ -11311,14 +11383,14 @@
       <c r="H142" s="17"/>
       <c r="I142" s="17"/>
     </row>
-    <row r="145" spans="3:9">
-      <c r="C145" s="17"/>
-      <c r="D145" s="17"/>
-      <c r="E145" s="17"/>
-      <c r="F145" s="17"/>
-      <c r="G145" s="17"/>
-      <c r="H145" s="17"/>
-      <c r="I145" s="17"/>
+    <row r="143" spans="3:9">
+      <c r="C143" s="17"/>
+      <c r="D143" s="17"/>
+      <c r="E143" s="17"/>
+      <c r="F143" s="17"/>
+      <c r="G143" s="17"/>
+      <c r="H143" s="17"/>
+      <c r="I143" s="17"/>
     </row>
     <row r="146" spans="3:9">
       <c r="C146" s="17"/>
@@ -11419,10 +11491,19 @@
       <c r="H156" s="17"/>
       <c r="I156" s="17"/>
     </row>
+    <row r="157" spans="3:9">
+      <c r="C157" s="17"/>
+      <c r="D157" s="17"/>
+      <c r="E157" s="17"/>
+      <c r="F157" s="17"/>
+      <c r="G157" s="17"/>
+      <c r="H157" s="17"/>
+      <c r="I157" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B123:I123"/>
+    <mergeCell ref="B124:I124"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
auto: actualizar indicadores adelantados 2026-07-27
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
+++ b/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PARA LA WEB - ABRIL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PAGINA WEB MAYO\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Índice" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Índice!$1:$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="38">
   <si>
     <t>DOMÉSTICO</t>
   </si>
@@ -1099,7 +1099,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="B1:W168"/>
+  <dimension ref="B1:W169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -4533,25 +4533,25 @@
         <v>33</v>
       </c>
       <c r="C132" s="10">
-        <v>130.79537920294501</v>
+        <v>127.91637176646699</v>
       </c>
       <c r="D132" s="10">
-        <v>131.77926673946001</v>
+        <v>129.76074747998001</v>
       </c>
       <c r="E132" s="10">
-        <v>122.510722209119</v>
+        <v>121.835541900515</v>
       </c>
       <c r="F132" s="10">
-        <v>175.89263798508301</v>
+        <v>178.26089135115899</v>
       </c>
       <c r="G132" s="10">
-        <v>115.221935986085</v>
+        <v>116.28415571143201</v>
       </c>
       <c r="H132" s="10">
-        <v>159.40834080794701</v>
+        <v>159.70014058565201</v>
       </c>
       <c r="I132" s="10">
-        <v>131.85001427717</v>
+        <v>130.23158135861601</v>
       </c>
     </row>
     <row r="133" spans="2:9">
@@ -4559,25 +4559,25 @@
         <v>6</v>
       </c>
       <c r="C133" s="12">
-        <v>133.81745310174699</v>
+        <v>133.72844868439199</v>
       </c>
       <c r="D133" s="12">
-        <v>130.33319574657801</v>
+        <v>130.28602618683101</v>
       </c>
       <c r="E133" s="12">
-        <v>117.55876343064899</v>
+        <v>117.548895332529</v>
       </c>
       <c r="F133" s="12">
         <v>171.086962259134</v>
       </c>
       <c r="G133" s="12">
-        <v>115.76923599584499</v>
+        <v>115.701034494035</v>
       </c>
       <c r="H133" s="12">
-        <v>153.05492493059</v>
+        <v>153.002938913702</v>
       </c>
       <c r="I133" s="12">
-        <v>131.28751996418501</v>
+        <v>131.231778811693</v>
       </c>
     </row>
     <row r="134" spans="2:9">
@@ -4585,25 +4585,25 @@
         <v>7</v>
       </c>
       <c r="C134" s="12">
-        <v>130.45201169262</v>
+        <v>130.365549430709</v>
       </c>
       <c r="D134" s="12">
-        <v>130.91666595341499</v>
+        <v>130.840996695846</v>
       </c>
       <c r="E134" s="12">
-        <v>117.182631524885</v>
+        <v>117.18309199657099</v>
       </c>
       <c r="F134" s="12">
         <v>173.441249375523</v>
       </c>
       <c r="G134" s="12">
-        <v>100.515598973637</v>
+        <v>100.509515157297</v>
       </c>
       <c r="H134" s="12">
-        <v>153.79914306051501</v>
+        <v>153.74872483915101</v>
       </c>
       <c r="I134" s="12">
-        <v>129.276682334128</v>
+        <v>129.21967342105299</v>
       </c>
     </row>
     <row r="135" spans="2:9">
@@ -4633,87 +4633,104 @@
       </c>
     </row>
     <row r="136" spans="2:9">
-      <c r="B136" s="33" t="s">
+      <c r="B136" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C136" s="16">
+      <c r="C136" s="12">
         <v>130.06703932590801</v>
       </c>
-      <c r="D136" s="16">
+      <c r="D136" s="12">
         <v>135.09744418304999</v>
       </c>
-      <c r="E136" s="16">
+      <c r="E136" s="12">
         <v>130.94791723485801</v>
       </c>
-      <c r="F136" s="16">
+      <c r="F136" s="12">
         <v>191.016110680964</v>
       </c>
-      <c r="G136" s="16">
+      <c r="G136" s="12">
         <v>131.75569020193799</v>
       </c>
-      <c r="H136" s="16">
+      <c r="H136" s="12">
         <v>161.88302648092599</v>
       </c>
-      <c r="I136" s="16">
+      <c r="I136" s="12">
         <v>135.904751935305</v>
       </c>
     </row>
-    <row r="137" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B137" s="29" t="s">
+    <row r="137" spans="2:9">
+      <c r="B137" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C137" s="16">
+        <v>116.575808699818</v>
+      </c>
+      <c r="D137" s="16">
+        <v>121.809509259378</v>
+      </c>
+      <c r="E137" s="16">
+        <v>119.14422829253201</v>
+      </c>
+      <c r="F137" s="16">
+        <v>187.73390481546099</v>
+      </c>
+      <c r="G137" s="16">
+        <v>120.60731993097301</v>
+      </c>
+      <c r="H137" s="16">
+        <v>160.96974393472399</v>
+      </c>
+      <c r="I137" s="16">
+        <v>123.870599749965</v>
+      </c>
+    </row>
+    <row r="138" spans="2:9" ht="14.25" customHeight="1">
+      <c r="B138" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C137" s="30"/>
-      <c r="D137" s="30"/>
-      <c r="E137" s="30"/>
-      <c r="F137" s="30"/>
-      <c r="G137" s="30"/>
-      <c r="H137" s="30"/>
-      <c r="I137" s="30"/>
-    </row>
-    <row r="138" spans="2:9" ht="34.5" customHeight="1">
-      <c r="B138" s="35" t="s">
+      <c r="C138" s="30"/>
+      <c r="D138" s="30"/>
+      <c r="E138" s="30"/>
+      <c r="F138" s="30"/>
+      <c r="G138" s="30"/>
+      <c r="H138" s="30"/>
+      <c r="I138" s="30"/>
+    </row>
+    <row r="139" spans="2:9" ht="34.5" customHeight="1">
+      <c r="B139" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C138" s="35"/>
-      <c r="D138" s="35"/>
-      <c r="E138" s="35"/>
-      <c r="F138" s="35"/>
-      <c r="G138" s="35"/>
-      <c r="H138" s="35"/>
-      <c r="I138" s="35"/>
-    </row>
-    <row r="139" spans="2:9">
-      <c r="B139" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C139" s="32"/>
-      <c r="D139" s="32"/>
-      <c r="E139" s="32"/>
-      <c r="F139" s="32"/>
-      <c r="G139" s="32"/>
-      <c r="H139" s="32"/>
-      <c r="I139" s="32"/>
+      <c r="C139" s="35"/>
+      <c r="D139" s="35"/>
+      <c r="E139" s="35"/>
+      <c r="F139" s="35"/>
+      <c r="G139" s="35"/>
+      <c r="H139" s="35"/>
+      <c r="I139" s="35"/>
     </row>
     <row r="140" spans="2:9">
       <c r="B140" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C140" s="32"/>
+      <c r="D140" s="32"/>
+      <c r="E140" s="32"/>
+      <c r="F140" s="32"/>
+      <c r="G140" s="32"/>
+      <c r="H140" s="32"/>
+      <c r="I140" s="32"/>
+    </row>
+    <row r="141" spans="2:9">
+      <c r="B141" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C140" s="30"/>
-      <c r="D140" s="30"/>
-      <c r="E140" s="30"/>
-      <c r="F140" s="30"/>
-      <c r="G140" s="30"/>
-      <c r="H140" s="30"/>
-      <c r="I140" s="30"/>
-    </row>
-    <row r="142" spans="2:9">
-      <c r="C142" s="17"/>
-      <c r="D142" s="17"/>
-      <c r="E142" s="17"/>
-      <c r="F142" s="17"/>
-      <c r="G142" s="17"/>
-      <c r="H142" s="17"/>
-      <c r="I142" s="17"/>
+      <c r="C141" s="30"/>
+      <c r="D141" s="30"/>
+      <c r="E141" s="30"/>
+      <c r="F141" s="30"/>
+      <c r="G141" s="30"/>
+      <c r="H141" s="30"/>
+      <c r="I141" s="30"/>
     </row>
     <row r="143" spans="2:9">
       <c r="C143" s="17"/>
@@ -4869,13 +4886,13 @@
       <c r="I159" s="17"/>
     </row>
     <row r="160" spans="3:9">
-      <c r="C160" s="18"/>
-      <c r="D160" s="18"/>
-      <c r="E160" s="18"/>
-      <c r="F160" s="18"/>
-      <c r="G160" s="18"/>
-      <c r="H160" s="18"/>
-      <c r="I160" s="18"/>
+      <c r="C160" s="17"/>
+      <c r="D160" s="17"/>
+      <c r="E160" s="17"/>
+      <c r="F160" s="17"/>
+      <c r="G160" s="17"/>
+      <c r="H160" s="17"/>
+      <c r="I160" s="17"/>
     </row>
     <row r="161" spans="3:9">
       <c r="C161" s="18"/>
@@ -4949,10 +4966,19 @@
       <c r="H168" s="18"/>
       <c r="I168" s="18"/>
     </row>
+    <row r="169" spans="3:9">
+      <c r="C169" s="18"/>
+      <c r="D169" s="18"/>
+      <c r="E169" s="18"/>
+      <c r="F169" s="18"/>
+      <c r="G169" s="18"/>
+      <c r="H169" s="18"/>
+      <c r="I169" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B138:I138"/>
+    <mergeCell ref="B139:I139"/>
     <mergeCell ref="B3:G3"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
@@ -4965,7 +4991,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja3"/>
-  <dimension ref="B1:K148"/>
+  <dimension ref="B1:K149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -7827,25 +7853,25 @@
         <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>4.6754931053025501</v>
+        <v>3.8753818831876998</v>
       </c>
       <c r="D118" s="10">
-        <v>3.6364812084440001</v>
+        <v>2.8974827418927398</v>
       </c>
       <c r="E118" s="10">
-        <v>-2.9324445375819299</v>
+        <v>-5.4740031709967401</v>
       </c>
       <c r="F118" s="10">
-        <v>16.038477753051101</v>
+        <v>15.891423486135199</v>
       </c>
       <c r="G118" s="10">
-        <v>1.8537277247402799</v>
+        <v>1.12210593068598</v>
       </c>
       <c r="H118" s="10">
-        <v>5.9368459809194301</v>
+        <v>5.5669924645801396</v>
       </c>
       <c r="I118" s="10">
-        <v>3.7909082765206801</v>
+        <v>2.7555741212210001</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
@@ -7855,25 +7881,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>7.3000843336288801</v>
+        <v>7.2287170996327799</v>
       </c>
       <c r="D119" s="12">
-        <v>0.33814940313814401</v>
+        <v>0.30183550546922799</v>
       </c>
       <c r="E119" s="12">
-        <v>-8.9783131613286002</v>
+        <v>-8.9859536885898201</v>
       </c>
       <c r="F119" s="12">
         <v>-11.3296548989108</v>
       </c>
       <c r="G119" s="12">
-        <v>5.1591213604943702</v>
+        <v>5.0971704462982297</v>
       </c>
       <c r="H119" s="12">
-        <v>-10.719053577852801</v>
+        <v>-10.749378383085601</v>
       </c>
       <c r="I119" s="12">
-        <v>0.45521916229560599</v>
+        <v>0.41256857607452302</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
@@ -7883,25 +7909,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-2.5149495309616499</v>
+        <v>-2.51472239958377</v>
       </c>
       <c r="D120" s="12">
-        <v>0.44767582310429899</v>
+        <v>0.42596318673466799</v>
       </c>
       <c r="E120" s="12">
-        <v>-0.31995224752927598</v>
+        <v>-0.31119249136523103</v>
       </c>
       <c r="F120" s="12">
         <v>1.37607628617773</v>
       </c>
       <c r="G120" s="12">
-        <v>-13.175898494099799</v>
+        <v>-13.129977102772999</v>
       </c>
       <c r="H120" s="12">
-        <v>0.48624252389308797</v>
+        <v>0.48743241845150598</v>
       </c>
       <c r="I120" s="12">
-        <v>-1.5316289245204699</v>
+        <v>-1.53324553614985</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
@@ -7911,121 +7937,140 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>-1.23186985027123</v>
+        <v>-1.1663639250119699</v>
       </c>
       <c r="D121" s="12">
-        <v>-0.112212511332987</v>
+        <v>-5.4444419448140803E-2</v>
       </c>
       <c r="E121" s="12">
-        <v>6.1194607322641001</v>
+        <v>6.1190437351855298</v>
       </c>
       <c r="F121" s="12">
         <v>-3.12210605626229</v>
       </c>
       <c r="G121" s="12">
-        <v>12.268364239182899</v>
+        <v>12.275159815778601</v>
       </c>
       <c r="H121" s="12">
-        <v>9.8161312207695897</v>
+        <v>9.8521427975745794</v>
       </c>
       <c r="I121" s="12">
-        <v>1.2797517008208401</v>
+        <v>1.3244341273289899</v>
       </c>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
     </row>
     <row r="122" spans="2:11">
-      <c r="B122" s="33" t="s">
+      <c r="B122" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C122" s="16">
+      <c r="C122" s="12">
         <v>0.94844698205578404</v>
       </c>
-      <c r="D122" s="16">
+      <c r="D122" s="12">
         <v>3.3093913093407399</v>
       </c>
-      <c r="E122" s="16">
+      <c r="E122" s="12">
         <v>5.3028957965092403</v>
       </c>
-      <c r="F122" s="16">
+      <c r="F122" s="12">
         <v>13.682316807083801</v>
       </c>
-      <c r="G122" s="16">
+      <c r="G122" s="12">
         <v>16.755815193875701</v>
       </c>
-      <c r="H122" s="16">
+      <c r="H122" s="12">
         <v>-4.1523962194836797</v>
       </c>
-      <c r="I122" s="16">
+      <c r="I122" s="12">
         <v>3.7986765184335298</v>
       </c>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
     </row>
-    <row r="123" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B123" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C123" s="30"/>
-      <c r="D123" s="30"/>
-      <c r="E123" s="30"/>
-      <c r="F123" s="30"/>
-      <c r="G123" s="30"/>
-      <c r="H123" s="30"/>
-      <c r="I123" s="30"/>
+    <row r="123" spans="2:11">
+      <c r="B123" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C123" s="16">
+        <v>-10.372520737006401</v>
+      </c>
+      <c r="D123" s="16">
+        <v>-9.8358151806833796</v>
+      </c>
+      <c r="E123" s="16">
+        <v>-9.0140333588935899</v>
+      </c>
+      <c r="F123" s="16">
+        <v>-1.7182874542895901</v>
+      </c>
+      <c r="G123" s="16">
+        <v>-8.4613956739772007</v>
+      </c>
+      <c r="H123" s="16">
+        <v>-0.56416201627460505</v>
+      </c>
+      <c r="I123" s="16">
+        <v>-8.85484283218344</v>
+      </c>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
     </row>
-    <row r="124" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B124" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C124" s="35"/>
-      <c r="D124" s="35"/>
-      <c r="E124" s="35"/>
-      <c r="F124" s="35"/>
-      <c r="G124" s="35"/>
-      <c r="H124" s="35"/>
-      <c r="I124" s="35"/>
+    <row r="124" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B124" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C124" s="30"/>
+      <c r="D124" s="30"/>
+      <c r="E124" s="30"/>
+      <c r="F124" s="30"/>
+      <c r="G124" s="30"/>
+      <c r="H124" s="30"/>
+      <c r="I124" s="30"/>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
     </row>
-    <row r="125" spans="2:11">
-      <c r="B125" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C125" s="32"/>
-      <c r="D125" s="32"/>
-      <c r="E125" s="32"/>
-      <c r="F125" s="32"/>
-      <c r="G125" s="32"/>
-      <c r="H125" s="32"/>
-      <c r="I125" s="32"/>
+    <row r="125" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B125" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C125" s="35"/>
+      <c r="D125" s="35"/>
+      <c r="E125" s="35"/>
+      <c r="F125" s="35"/>
+      <c r="G125" s="35"/>
+      <c r="H125" s="35"/>
+      <c r="I125" s="35"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
     </row>
     <row r="126" spans="2:11">
       <c r="B126" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
-      <c r="E126" s="30"/>
-      <c r="F126" s="30"/>
-      <c r="G126" s="30"/>
-      <c r="H126" s="30"/>
-      <c r="I126" s="30"/>
+        <v>24</v>
+      </c>
+      <c r="C126" s="32"/>
+      <c r="D126" s="32"/>
+      <c r="E126" s="32"/>
+      <c r="F126" s="32"/>
+      <c r="G126" s="32"/>
+      <c r="H126" s="32"/>
+      <c r="I126" s="32"/>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
     </row>
     <row r="127" spans="2:11">
-      <c r="C127" s="19"/>
-      <c r="D127" s="19"/>
-      <c r="E127" s="19"/>
-      <c r="F127" s="19"/>
-      <c r="G127" s="19"/>
-      <c r="H127" s="19"/>
-      <c r="I127" s="19"/>
+      <c r="B127" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C127" s="30"/>
+      <c r="D127" s="30"/>
+      <c r="E127" s="30"/>
+      <c r="F127" s="30"/>
+      <c r="G127" s="30"/>
+      <c r="H127" s="30"/>
+      <c r="I127" s="30"/>
+      <c r="J127" s="1"/>
+      <c r="K127" s="1"/>
     </row>
     <row r="128" spans="2:11">
       <c r="C128" s="19"/>
@@ -8064,13 +8109,13 @@
       <c r="I131" s="19"/>
     </row>
     <row r="132" spans="3:9">
-      <c r="C132" s="17"/>
-      <c r="D132" s="17"/>
-      <c r="E132" s="17"/>
-      <c r="F132" s="17"/>
-      <c r="G132" s="17"/>
-      <c r="H132" s="17"/>
-      <c r="I132" s="17"/>
+      <c r="C132" s="19"/>
+      <c r="D132" s="19"/>
+      <c r="E132" s="19"/>
+      <c r="F132" s="19"/>
+      <c r="G132" s="19"/>
+      <c r="H132" s="19"/>
+      <c r="I132" s="19"/>
     </row>
     <row r="133" spans="3:9">
       <c r="C133" s="17"/>
@@ -8216,10 +8261,19 @@
       <c r="H148" s="17"/>
       <c r="I148" s="17"/>
     </row>
+    <row r="149" spans="3:9">
+      <c r="C149" s="17"/>
+      <c r="D149" s="17"/>
+      <c r="E149" s="17"/>
+      <c r="F149" s="17"/>
+      <c r="G149" s="17"/>
+      <c r="H149" s="17"/>
+      <c r="I149" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B124:I124"/>
+    <mergeCell ref="B125:I125"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8231,7 +8285,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="B1:K157"/>
+  <dimension ref="B1:K158"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -11093,25 +11147,25 @@
         <v>37</v>
       </c>
       <c r="C118" s="10">
-        <v>4.6754931053025501</v>
+        <v>3.8753818831876998</v>
       </c>
       <c r="D118" s="10">
-        <v>3.6364812084440001</v>
+        <v>2.8974827418927398</v>
       </c>
       <c r="E118" s="10">
-        <v>-2.9324445375819299</v>
+        <v>-5.4740031709967401</v>
       </c>
       <c r="F118" s="10">
-        <v>16.038477753051101</v>
+        <v>15.891423486135199</v>
       </c>
       <c r="G118" s="10">
-        <v>1.8537277247402799</v>
+        <v>1.12210593068598</v>
       </c>
       <c r="H118" s="10">
-        <v>5.9368459809194301</v>
+        <v>5.5669924645801396</v>
       </c>
       <c r="I118" s="10">
-        <v>3.7909082765206801</v>
+        <v>2.7555741212210001</v>
       </c>
       <c r="K118" s="1"/>
     </row>
@@ -11120,25 +11174,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>3.72865534857034</v>
+        <v>3.6596635368272499</v>
       </c>
       <c r="D119" s="12">
-        <v>2.7661129814063901</v>
+        <v>2.7289203669039499</v>
       </c>
       <c r="E119" s="12">
-        <v>-2.5515743658463301</v>
+        <v>-2.5597543653440402</v>
       </c>
       <c r="F119" s="12">
         <v>13.293318580951601</v>
       </c>
       <c r="G119" s="12">
-        <v>6.0160708382844801</v>
+        <v>5.9536150814947204</v>
       </c>
       <c r="H119" s="12">
-        <v>-5.2608625487796203</v>
+        <v>-5.2930412611058903</v>
       </c>
       <c r="I119" s="12">
-        <v>2.9187034942509</v>
+        <v>2.8750069787910801</v>
       </c>
       <c r="K119" s="1"/>
     </row>
@@ -11147,25 +11201,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-1.0685583386863899</v>
+        <v>-1.1341290884900299</v>
       </c>
       <c r="D120" s="12">
-        <v>-0.36138624519996798</v>
+        <v>-0.41897692605847903</v>
       </c>
       <c r="E120" s="12">
-        <v>-6.3351241779361596</v>
+        <v>-6.3347561197798603</v>
       </c>
       <c r="F120" s="12">
         <v>14.561465258757099</v>
       </c>
       <c r="G120" s="12">
-        <v>-6.4747464267629802</v>
+        <v>-6.4804071448178897</v>
       </c>
       <c r="H120" s="12">
-        <v>4.9140774905373803</v>
+        <v>4.8796847034395796</v>
       </c>
       <c r="I120" s="12">
-        <v>-0.82182133461548001</v>
+        <v>-0.86555729739281595</v>
       </c>
       <c r="K120" s="1"/>
     </row>
@@ -11197,92 +11251,110 @@
       <c r="K121" s="1"/>
     </row>
     <row r="122" spans="2:11">
-      <c r="B122" s="33" t="s">
+      <c r="B122" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C122" s="16">
+      <c r="C122" s="12">
         <v>16.1802925760467</v>
       </c>
-      <c r="D122" s="16">
+      <c r="D122" s="12">
         <v>11.9746416696604</v>
       </c>
-      <c r="E122" s="16">
+      <c r="E122" s="12">
         <v>-5.6614115014834798</v>
       </c>
-      <c r="F122" s="16">
+      <c r="F122" s="12">
         <v>16.714827162760098</v>
       </c>
-      <c r="G122" s="16">
+      <c r="G122" s="12">
         <v>9.49079036829648</v>
       </c>
-      <c r="H122" s="16">
+      <c r="H122" s="12">
         <v>6.5290642010867197</v>
       </c>
-      <c r="I122" s="16">
+      <c r="I122" s="12">
         <v>10.200452758813</v>
       </c>
       <c r="K122" s="1"/>
     </row>
-    <row r="123" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B123" s="29" t="s">
+    <row r="123" spans="2:11">
+      <c r="B123" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C123" s="16">
+        <v>0.57655280366217798</v>
+      </c>
+      <c r="D123" s="16">
+        <v>-8.4861005177705506E-2</v>
+      </c>
+      <c r="E123" s="16">
+        <v>-14.657993796920801</v>
+      </c>
+      <c r="F123" s="16">
+        <v>15.343608282550001</v>
+      </c>
+      <c r="G123" s="16">
+        <v>-1.5204325546550701</v>
+      </c>
+      <c r="H123" s="16">
+        <v>4.1923386316592</v>
+      </c>
+      <c r="I123" s="16">
+        <v>-1.34462621765121</v>
+      </c>
+      <c r="K123" s="1"/>
+    </row>
+    <row r="124" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B124" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C123" s="30"/>
-      <c r="D123" s="30"/>
-      <c r="E123" s="30"/>
-      <c r="F123" s="30"/>
-      <c r="G123" s="30"/>
-      <c r="H123" s="30"/>
-      <c r="I123" s="30"/>
-      <c r="K123" s="1"/>
-    </row>
-    <row r="124" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B124" s="35" t="s">
+      <c r="C124" s="30"/>
+      <c r="D124" s="30"/>
+      <c r="E124" s="30"/>
+      <c r="F124" s="30"/>
+      <c r="G124" s="30"/>
+      <c r="H124" s="30"/>
+      <c r="I124" s="30"/>
+      <c r="K124" s="1"/>
+    </row>
+    <row r="125" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B125" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C124" s="35"/>
-      <c r="D124" s="35"/>
-      <c r="E124" s="35"/>
-      <c r="F124" s="35"/>
-      <c r="G124" s="35"/>
-      <c r="H124" s="35"/>
-      <c r="I124" s="35"/>
-      <c r="K124" s="1"/>
-    </row>
-    <row r="125" spans="2:11">
-      <c r="B125" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C125" s="32"/>
-      <c r="D125" s="32"/>
-      <c r="E125" s="32"/>
-      <c r="F125" s="32"/>
-      <c r="G125" s="32"/>
-      <c r="H125" s="32"/>
-      <c r="I125" s="32"/>
+      <c r="C125" s="35"/>
+      <c r="D125" s="35"/>
+      <c r="E125" s="35"/>
+      <c r="F125" s="35"/>
+      <c r="G125" s="35"/>
+      <c r="H125" s="35"/>
+      <c r="I125" s="35"/>
       <c r="K125" s="1"/>
     </row>
     <row r="126" spans="2:11">
       <c r="B126" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C126" s="32"/>
+      <c r="D126" s="32"/>
+      <c r="E126" s="32"/>
+      <c r="F126" s="32"/>
+      <c r="G126" s="32"/>
+      <c r="H126" s="32"/>
+      <c r="I126" s="32"/>
+      <c r="K126" s="1"/>
+    </row>
+    <row r="127" spans="2:11">
+      <c r="B127" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
-      <c r="E126" s="30"/>
-      <c r="F126" s="30"/>
-      <c r="G126" s="30"/>
-      <c r="H126" s="30"/>
-      <c r="I126" s="30"/>
-      <c r="K126" s="1"/>
-    </row>
-    <row r="131" spans="3:9">
-      <c r="C131" s="17"/>
-      <c r="D131" s="17"/>
-      <c r="E131" s="17"/>
-      <c r="F131" s="17"/>
-      <c r="G131" s="17"/>
-      <c r="H131" s="17"/>
-      <c r="I131" s="17"/>
+      <c r="C127" s="30"/>
+      <c r="D127" s="30"/>
+      <c r="E127" s="30"/>
+      <c r="F127" s="30"/>
+      <c r="G127" s="30"/>
+      <c r="H127" s="30"/>
+      <c r="I127" s="30"/>
+      <c r="K127" s="1"/>
     </row>
     <row r="132" spans="3:9">
       <c r="C132" s="17"/>
@@ -11392,14 +11464,14 @@
       <c r="H143" s="17"/>
       <c r="I143" s="17"/>
     </row>
-    <row r="146" spans="3:9">
-      <c r="C146" s="17"/>
-      <c r="D146" s="17"/>
-      <c r="E146" s="17"/>
-      <c r="F146" s="17"/>
-      <c r="G146" s="17"/>
-      <c r="H146" s="17"/>
-      <c r="I146" s="17"/>
+    <row r="144" spans="3:9">
+      <c r="C144" s="17"/>
+      <c r="D144" s="17"/>
+      <c r="E144" s="17"/>
+      <c r="F144" s="17"/>
+      <c r="G144" s="17"/>
+      <c r="H144" s="17"/>
+      <c r="I144" s="17"/>
     </row>
     <row r="147" spans="3:9">
       <c r="C147" s="17"/>
@@ -11500,10 +11572,19 @@
       <c r="H157" s="17"/>
       <c r="I157" s="17"/>
     </row>
+    <row r="158" spans="3:9">
+      <c r="C158" s="17"/>
+      <c r="D158" s="17"/>
+      <c r="E158" s="17"/>
+      <c r="F158" s="17"/>
+      <c r="G158" s="17"/>
+      <c r="H158" s="17"/>
+      <c r="I158" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B124:I124"/>
+    <mergeCell ref="B125:I125"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
auto: actualizar indicadores adelantados 2026-08-24
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
+++ b/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PAGINA WEB MAYO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\csoraide\Desktop\PAGINA WEB JUNIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
   </bookViews>
   <sheets>
     <sheet name="Índice" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="38">
   <si>
     <t>DOMÉSTICO</t>
   </si>
@@ -1099,7 +1099,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="B1:W169"/>
+  <dimension ref="B1:W170"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -4533,25 +4533,25 @@
         <v>33</v>
       </c>
       <c r="C132" s="10">
-        <v>127.91637176646699</v>
+        <v>125.145180201377</v>
       </c>
       <c r="D132" s="10">
-        <v>129.76074747998001</v>
+        <v>126.899692551635</v>
       </c>
       <c r="E132" s="10">
-        <v>121.835541900515</v>
+        <v>118.274828201093</v>
       </c>
       <c r="F132" s="10">
-        <v>178.26089135115899</v>
+        <v>180.94476445483599</v>
       </c>
       <c r="G132" s="10">
-        <v>116.28415571143201</v>
+        <v>116.691000897694</v>
       </c>
       <c r="H132" s="10">
-        <v>159.70014058565201</v>
+        <v>160.687613248579</v>
       </c>
       <c r="I132" s="10">
-        <v>130.23158135861601</v>
+        <v>127.89020849115001</v>
       </c>
     </row>
     <row r="133" spans="2:9">
@@ -4559,25 +4559,25 @@
         <v>6</v>
       </c>
       <c r="C133" s="12">
-        <v>133.72844868439199</v>
+        <v>133.81745310174699</v>
       </c>
       <c r="D133" s="12">
-        <v>130.28602618683101</v>
+        <v>130.315067629449</v>
       </c>
       <c r="E133" s="12">
-        <v>117.548895332529</v>
+        <v>117.55876343064899</v>
       </c>
       <c r="F133" s="12">
         <v>171.086962259134</v>
       </c>
       <c r="G133" s="12">
-        <v>115.701034494035</v>
+        <v>115.76923599584499</v>
       </c>
       <c r="H133" s="12">
-        <v>153.002938913702</v>
+        <v>152.85179416885401</v>
       </c>
       <c r="I133" s="12">
-        <v>131.231778811693</v>
+        <v>131.275379933279</v>
       </c>
     </row>
     <row r="134" spans="2:9">
@@ -4585,25 +4585,25 @@
         <v>7</v>
       </c>
       <c r="C134" s="12">
-        <v>130.365549430709</v>
+        <v>130.45201169262</v>
       </c>
       <c r="D134" s="12">
-        <v>130.840996695846</v>
+        <v>130.87266117091599</v>
       </c>
       <c r="E134" s="12">
-        <v>117.18309199657099</v>
+        <v>117.192635509624</v>
       </c>
       <c r="F134" s="12">
         <v>173.441249375523</v>
       </c>
       <c r="G134" s="12">
-        <v>100.509515157297</v>
+        <v>100.571432663838</v>
       </c>
       <c r="H134" s="12">
-        <v>153.74872483915101</v>
+        <v>153.57623840542101</v>
       </c>
       <c r="I134" s="12">
-        <v>129.21967342105299</v>
+        <v>129.26183797899</v>
       </c>
     </row>
     <row r="135" spans="2:9">
@@ -4614,7 +4614,7 @@
         <v>128.84501269150601</v>
       </c>
       <c r="D135" s="12">
-        <v>130.76976107479501</v>
+        <v>130.74387424263199</v>
       </c>
       <c r="E135" s="12">
         <v>124.35357664608399</v>
@@ -4626,10 +4626,10 @@
         <v>112.84721877291901</v>
       </c>
       <c r="H135" s="12">
-        <v>168.896268759755</v>
+        <v>168.68080390186901</v>
       </c>
       <c r="I135" s="12">
-        <v>130.931102875064</v>
+        <v>130.91635057244599</v>
       </c>
     </row>
     <row r="136" spans="2:9">
@@ -4640,7 +4640,7 @@
         <v>130.06703932590801</v>
       </c>
       <c r="D136" s="12">
-        <v>135.09744418304999</v>
+        <v>135.09732653873701</v>
       </c>
       <c r="E136" s="12">
         <v>130.94791723485801</v>
@@ -4652,94 +4652,111 @@
         <v>131.75569020193799</v>
       </c>
       <c r="H136" s="12">
-        <v>161.88302648092599</v>
+        <v>161.671217884187</v>
       </c>
       <c r="I136" s="12">
-        <v>135.904751935305</v>
+        <v>135.89738379486101</v>
       </c>
     </row>
     <row r="137" spans="2:9">
-      <c r="B137" s="33" t="s">
+      <c r="B137" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C137" s="16">
+      <c r="C137" s="12">
         <v>116.575808699818</v>
       </c>
-      <c r="D137" s="16">
-        <v>121.809509259378</v>
-      </c>
-      <c r="E137" s="16">
+      <c r="D137" s="12">
+        <v>121.813157685467</v>
+      </c>
+      <c r="E137" s="12">
         <v>119.14422829253201</v>
       </c>
-      <c r="F137" s="16">
+      <c r="F137" s="12">
         <v>187.73390481546099</v>
       </c>
-      <c r="G137" s="16">
+      <c r="G137" s="12">
         <v>120.60731993097301</v>
       </c>
-      <c r="H137" s="16">
-        <v>160.96974393472399</v>
-      </c>
-      <c r="I137" s="16">
-        <v>123.870599749965</v>
-      </c>
-    </row>
-    <row r="138" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B138" s="29" t="s">
+      <c r="H137" s="12">
+        <v>160.94685180598799</v>
+      </c>
+      <c r="I137" s="12">
+        <v>123.870834517403</v>
+      </c>
+    </row>
+    <row r="138" spans="2:9">
+      <c r="B138" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C138" s="16">
+        <v>111.113755696665</v>
+      </c>
+      <c r="D138" s="16">
+        <v>112.556068042611</v>
+      </c>
+      <c r="E138" s="16">
+        <v>100.45184809281</v>
+      </c>
+      <c r="F138" s="16">
+        <v>194.36412997321901</v>
+      </c>
+      <c r="G138" s="16">
+        <v>118.59510782065399</v>
+      </c>
+      <c r="H138" s="16">
+        <v>166.39877332515599</v>
+      </c>
+      <c r="I138" s="16">
+        <v>116.119464149923</v>
+      </c>
+    </row>
+    <row r="139" spans="2:9" ht="14.25" customHeight="1">
+      <c r="B139" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C138" s="30"/>
-      <c r="D138" s="30"/>
-      <c r="E138" s="30"/>
-      <c r="F138" s="30"/>
-      <c r="G138" s="30"/>
-      <c r="H138" s="30"/>
-      <c r="I138" s="30"/>
-    </row>
-    <row r="139" spans="2:9" ht="34.5" customHeight="1">
-      <c r="B139" s="35" t="s">
+      <c r="C139" s="30"/>
+      <c r="D139" s="30"/>
+      <c r="E139" s="30"/>
+      <c r="F139" s="30"/>
+      <c r="G139" s="30"/>
+      <c r="H139" s="30"/>
+      <c r="I139" s="30"/>
+    </row>
+    <row r="140" spans="2:9" ht="34.5" customHeight="1">
+      <c r="B140" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C139" s="35"/>
-      <c r="D139" s="35"/>
-      <c r="E139" s="35"/>
-      <c r="F139" s="35"/>
-      <c r="G139" s="35"/>
-      <c r="H139" s="35"/>
-      <c r="I139" s="35"/>
-    </row>
-    <row r="140" spans="2:9">
-      <c r="B140" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C140" s="32"/>
-      <c r="D140" s="32"/>
-      <c r="E140" s="32"/>
-      <c r="F140" s="32"/>
-      <c r="G140" s="32"/>
-      <c r="H140" s="32"/>
-      <c r="I140" s="32"/>
+      <c r="C140" s="35"/>
+      <c r="D140" s="35"/>
+      <c r="E140" s="35"/>
+      <c r="F140" s="35"/>
+      <c r="G140" s="35"/>
+      <c r="H140" s="35"/>
+      <c r="I140" s="35"/>
     </row>
     <row r="141" spans="2:9">
       <c r="B141" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C141" s="32"/>
+      <c r="D141" s="32"/>
+      <c r="E141" s="32"/>
+      <c r="F141" s="32"/>
+      <c r="G141" s="32"/>
+      <c r="H141" s="32"/>
+      <c r="I141" s="32"/>
+    </row>
+    <row r="142" spans="2:9">
+      <c r="B142" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C141" s="30"/>
-      <c r="D141" s="30"/>
-      <c r="E141" s="30"/>
-      <c r="F141" s="30"/>
-      <c r="G141" s="30"/>
-      <c r="H141" s="30"/>
-      <c r="I141" s="30"/>
-    </row>
-    <row r="143" spans="2:9">
-      <c r="C143" s="17"/>
-      <c r="D143" s="17"/>
-      <c r="E143" s="17"/>
-      <c r="F143" s="17"/>
-      <c r="G143" s="17"/>
-      <c r="H143" s="17"/>
-      <c r="I143" s="17"/>
+      <c r="C142" s="30"/>
+      <c r="D142" s="30"/>
+      <c r="E142" s="30"/>
+      <c r="F142" s="30"/>
+      <c r="G142" s="30"/>
+      <c r="H142" s="30"/>
+      <c r="I142" s="30"/>
     </row>
     <row r="144" spans="2:9">
       <c r="C144" s="17"/>
@@ -4895,13 +4912,13 @@
       <c r="I160" s="17"/>
     </row>
     <row r="161" spans="3:9">
-      <c r="C161" s="18"/>
-      <c r="D161" s="18"/>
-      <c r="E161" s="18"/>
-      <c r="F161" s="18"/>
-      <c r="G161" s="18"/>
-      <c r="H161" s="18"/>
-      <c r="I161" s="18"/>
+      <c r="C161" s="17"/>
+      <c r="D161" s="17"/>
+      <c r="E161" s="17"/>
+      <c r="F161" s="17"/>
+      <c r="G161" s="17"/>
+      <c r="H161" s="17"/>
+      <c r="I161" s="17"/>
     </row>
     <row r="162" spans="3:9">
       <c r="C162" s="18"/>
@@ -4975,10 +4992,19 @@
       <c r="H169" s="18"/>
       <c r="I169" s="18"/>
     </row>
+    <row r="170" spans="3:9">
+      <c r="C170" s="18"/>
+      <c r="D170" s="18"/>
+      <c r="E170" s="18"/>
+      <c r="F170" s="18"/>
+      <c r="G170" s="18"/>
+      <c r="H170" s="18"/>
+      <c r="I170" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B139:I139"/>
+    <mergeCell ref="B140:I140"/>
     <mergeCell ref="B3:G3"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
@@ -4991,7 +5017,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja3"/>
-  <dimension ref="B1:K149"/>
+  <dimension ref="B1:K150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -7853,25 +7879,25 @@
         <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>3.8753818831876998</v>
+        <v>3.6360074606287802</v>
       </c>
       <c r="D118" s="10">
-        <v>2.8974827418927398</v>
+        <v>1.8616319233407901</v>
       </c>
       <c r="E118" s="10">
-        <v>-5.4740031709967401</v>
+        <v>-8.3048776292568203</v>
       </c>
       <c r="F118" s="10">
-        <v>15.891423486135199</v>
+        <v>16.2847842921989</v>
       </c>
       <c r="G118" s="10">
-        <v>1.12210593068598</v>
+        <v>0.71257925509588904</v>
       </c>
       <c r="H118" s="10">
-        <v>5.5669924645801396</v>
+        <v>5.49063354222044</v>
       </c>
       <c r="I118" s="10">
-        <v>2.7555741212210001</v>
+        <v>1.87263882516264</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
@@ -7881,25 +7907,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>7.2287170996327799</v>
+        <v>7.3000843336288801</v>
       </c>
       <c r="D119" s="12">
-        <v>0.30183550546922799</v>
+        <v>0.32419331379016603</v>
       </c>
       <c r="E119" s="12">
-        <v>-8.9859536885898201</v>
+        <v>-8.9783131613286002</v>
       </c>
       <c r="F119" s="12">
         <v>-11.3296548989108</v>
       </c>
       <c r="G119" s="12">
-        <v>5.0971704462982297</v>
+        <v>5.1591213604943702</v>
       </c>
       <c r="H119" s="12">
-        <v>-10.749378383085601</v>
+        <v>-10.837545071435599</v>
       </c>
       <c r="I119" s="12">
-        <v>0.41256857607452302</v>
+        <v>0.44593016463887503</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
@@ -7909,25 +7935,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-2.51472239958377</v>
+        <v>-2.5149495309616499</v>
       </c>
       <c r="D120" s="12">
-        <v>0.42596318673466799</v>
+        <v>0.42788109741207497</v>
       </c>
       <c r="E120" s="12">
-        <v>-0.31119249136523103</v>
+        <v>-0.31144247382378598</v>
       </c>
       <c r="F120" s="12">
         <v>1.37607628617773</v>
       </c>
       <c r="G120" s="12">
-        <v>-13.129977102772999</v>
+        <v>-13.127670059558801</v>
       </c>
       <c r="H120" s="12">
-        <v>0.48743241845150598</v>
+        <v>0.47395206612104201</v>
       </c>
       <c r="I120" s="12">
-        <v>-1.53324553614985</v>
+        <v>-1.5338306050327</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
@@ -7937,25 +7963,25 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>-1.1663639250119699</v>
+        <v>-1.23186985027123</v>
       </c>
       <c r="D121" s="12">
-        <v>-5.4444419448140803E-2</v>
+        <v>-9.8406288319763405E-2</v>
       </c>
       <c r="E121" s="12">
-        <v>6.1190437351855298</v>
+        <v>6.11040199353834</v>
       </c>
       <c r="F121" s="12">
         <v>-3.12210605626229</v>
       </c>
       <c r="G121" s="12">
-        <v>12.275159815778601</v>
+        <v>12.2060368276878</v>
       </c>
       <c r="H121" s="12">
-        <v>9.8521427975745794</v>
+        <v>9.8352229832417297</v>
       </c>
       <c r="I121" s="12">
-        <v>1.3244341273289899</v>
+        <v>1.27996988076684</v>
       </c>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
@@ -7968,7 +7994,7 @@
         <v>0.94844698205578404</v>
       </c>
       <c r="D122" s="12">
-        <v>3.3093913093407399</v>
+        <v>3.3297562285986801</v>
       </c>
       <c r="E122" s="12">
         <v>5.3028957965092403</v>
@@ -7980,106 +8006,125 @@
         <v>16.755815193875701</v>
       </c>
       <c r="H122" s="12">
-        <v>-4.1523962194836797</v>
+        <v>-4.1555327313707</v>
       </c>
       <c r="I122" s="12">
-        <v>3.7986765184335298</v>
+        <v>3.80474493876015</v>
       </c>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
     </row>
     <row r="123" spans="2:11">
-      <c r="B123" s="33" t="s">
+      <c r="B123" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C123" s="16">
+      <c r="C123" s="12">
         <v>-10.372520737006401</v>
       </c>
-      <c r="D123" s="16">
-        <v>-9.8358151806833796</v>
-      </c>
-      <c r="E123" s="16">
+      <c r="D123" s="12">
+        <v>-9.8330360737828997</v>
+      </c>
+      <c r="E123" s="12">
         <v>-9.0140333588935899</v>
       </c>
-      <c r="F123" s="16">
+      <c r="F123" s="12">
         <v>-1.7182874542895901</v>
       </c>
-      <c r="G123" s="16">
+      <c r="G123" s="12">
         <v>-8.4613956739772007</v>
       </c>
-      <c r="H123" s="16">
-        <v>-0.56416201627460505</v>
-      </c>
-      <c r="I123" s="16">
-        <v>-8.85484283218344</v>
+      <c r="H123" s="12">
+        <v>-0.44804887825982098</v>
+      </c>
+      <c r="I123" s="12">
+        <v>-8.8497283329695406</v>
       </c>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
     </row>
-    <row r="124" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B124" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C124" s="30"/>
-      <c r="D124" s="30"/>
-      <c r="E124" s="30"/>
-      <c r="F124" s="30"/>
-      <c r="G124" s="30"/>
-      <c r="H124" s="30"/>
-      <c r="I124" s="30"/>
+    <row r="124" spans="2:11">
+      <c r="B124" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C124" s="16">
+        <v>-4.6854086315777401</v>
+      </c>
+      <c r="D124" s="16">
+        <v>-7.5994168600068397</v>
+      </c>
+      <c r="E124" s="16">
+        <v>-15.6888675747067</v>
+      </c>
+      <c r="F124" s="16">
+        <v>3.5317142975718201</v>
+      </c>
+      <c r="G124" s="16">
+        <v>-1.66839965556889</v>
+      </c>
+      <c r="H124" s="16">
+        <v>3.3874048842783302</v>
+      </c>
+      <c r="I124" s="16">
+        <v>-6.2576234330533502</v>
+      </c>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
     </row>
-    <row r="125" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B125" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C125" s="35"/>
-      <c r="D125" s="35"/>
-      <c r="E125" s="35"/>
-      <c r="F125" s="35"/>
-      <c r="G125" s="35"/>
-      <c r="H125" s="35"/>
-      <c r="I125" s="35"/>
+    <row r="125" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B125" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C125" s="30"/>
+      <c r="D125" s="30"/>
+      <c r="E125" s="30"/>
+      <c r="F125" s="30"/>
+      <c r="G125" s="30"/>
+      <c r="H125" s="30"/>
+      <c r="I125" s="30"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
     </row>
-    <row r="126" spans="2:11">
-      <c r="B126" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C126" s="32"/>
-      <c r="D126" s="32"/>
-      <c r="E126" s="32"/>
-      <c r="F126" s="32"/>
-      <c r="G126" s="32"/>
-      <c r="H126" s="32"/>
-      <c r="I126" s="32"/>
+    <row r="126" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B126" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C126" s="35"/>
+      <c r="D126" s="35"/>
+      <c r="E126" s="35"/>
+      <c r="F126" s="35"/>
+      <c r="G126" s="35"/>
+      <c r="H126" s="35"/>
+      <c r="I126" s="35"/>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
     </row>
     <row r="127" spans="2:11">
       <c r="B127" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C127" s="30"/>
-      <c r="D127" s="30"/>
-      <c r="E127" s="30"/>
-      <c r="F127" s="30"/>
-      <c r="G127" s="30"/>
-      <c r="H127" s="30"/>
-      <c r="I127" s="30"/>
+        <v>24</v>
+      </c>
+      <c r="C127" s="32"/>
+      <c r="D127" s="32"/>
+      <c r="E127" s="32"/>
+      <c r="F127" s="32"/>
+      <c r="G127" s="32"/>
+      <c r="H127" s="32"/>
+      <c r="I127" s="32"/>
       <c r="J127" s="1"/>
       <c r="K127" s="1"/>
     </row>
     <row r="128" spans="2:11">
-      <c r="C128" s="19"/>
-      <c r="D128" s="19"/>
-      <c r="E128" s="19"/>
-      <c r="F128" s="19"/>
-      <c r="G128" s="19"/>
-      <c r="H128" s="19"/>
-      <c r="I128" s="19"/>
+      <c r="B128" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C128" s="30"/>
+      <c r="D128" s="30"/>
+      <c r="E128" s="30"/>
+      <c r="F128" s="30"/>
+      <c r="G128" s="30"/>
+      <c r="H128" s="30"/>
+      <c r="I128" s="30"/>
+      <c r="J128" s="1"/>
+      <c r="K128" s="1"/>
     </row>
     <row r="129" spans="3:9">
       <c r="C129" s="19"/>
@@ -8118,13 +8163,13 @@
       <c r="I132" s="19"/>
     </row>
     <row r="133" spans="3:9">
-      <c r="C133" s="17"/>
-      <c r="D133" s="17"/>
-      <c r="E133" s="17"/>
-      <c r="F133" s="17"/>
-      <c r="G133" s="17"/>
-      <c r="H133" s="17"/>
-      <c r="I133" s="17"/>
+      <c r="C133" s="19"/>
+      <c r="D133" s="19"/>
+      <c r="E133" s="19"/>
+      <c r="F133" s="19"/>
+      <c r="G133" s="19"/>
+      <c r="H133" s="19"/>
+      <c r="I133" s="19"/>
     </row>
     <row r="134" spans="3:9">
       <c r="C134" s="17"/>
@@ -8270,10 +8315,19 @@
       <c r="H149" s="17"/>
       <c r="I149" s="17"/>
     </row>
+    <row r="150" spans="3:9">
+      <c r="C150" s="17"/>
+      <c r="D150" s="17"/>
+      <c r="E150" s="17"/>
+      <c r="F150" s="17"/>
+      <c r="G150" s="17"/>
+      <c r="H150" s="17"/>
+      <c r="I150" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B125:I125"/>
+    <mergeCell ref="B126:I126"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8285,7 +8339,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="B1:K158"/>
+  <dimension ref="B1:K159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -11147,25 +11201,25 @@
         <v>37</v>
       </c>
       <c r="C118" s="10">
-        <v>3.8753818831876998</v>
+        <v>3.6360074606287802</v>
       </c>
       <c r="D118" s="10">
-        <v>2.8974827418927398</v>
+        <v>1.8616319233407901</v>
       </c>
       <c r="E118" s="10">
-        <v>-5.4740031709967401</v>
+        <v>-8.3048776292568203</v>
       </c>
       <c r="F118" s="10">
-        <v>15.891423486135199</v>
+        <v>16.2847842921989</v>
       </c>
       <c r="G118" s="10">
-        <v>1.12210593068598</v>
+        <v>0.71257925509588904</v>
       </c>
       <c r="H118" s="10">
-        <v>5.5669924645801396</v>
+        <v>5.49063354222044</v>
       </c>
       <c r="I118" s="10">
-        <v>2.7555741212210001</v>
+        <v>1.87263882516264</v>
       </c>
       <c r="K118" s="1"/>
     </row>
@@ -11174,25 +11228,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>3.6596635368272499</v>
+        <v>3.72865534857034</v>
       </c>
       <c r="D119" s="12">
-        <v>2.7289203669039499</v>
+        <v>2.7518191852456502</v>
       </c>
       <c r="E119" s="12">
-        <v>-2.5597543653440402</v>
+        <v>-2.5515743658463301</v>
       </c>
       <c r="F119" s="12">
         <v>13.293318580951601</v>
       </c>
       <c r="G119" s="12">
-        <v>5.9536150814947204</v>
+        <v>6.0160708382844801</v>
       </c>
       <c r="H119" s="12">
-        <v>-5.2930412611058903</v>
+        <v>-5.3865980203131096</v>
       </c>
       <c r="I119" s="12">
-        <v>2.8750069787910801</v>
+        <v>2.9091867005634802</v>
       </c>
       <c r="K119" s="1"/>
     </row>
@@ -11201,25 +11255,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-1.1341290884900299</v>
+        <v>-1.0685583386863899</v>
       </c>
       <c r="D120" s="12">
-        <v>-0.41897692605847903</v>
+        <v>-0.39487759249986498</v>
       </c>
       <c r="E120" s="12">
-        <v>-6.3347561197798603</v>
+        <v>-6.3271279247704504</v>
       </c>
       <c r="F120" s="12">
         <v>14.561465258757099</v>
       </c>
       <c r="G120" s="12">
-        <v>-6.4804071448178897</v>
+        <v>-6.4227956839202101</v>
       </c>
       <c r="H120" s="12">
-        <v>4.8796847034395796</v>
+        <v>4.76202309158404</v>
       </c>
       <c r="I120" s="12">
-        <v>-0.86555729739281595</v>
+        <v>-0.83320959179789</v>
       </c>
       <c r="K120" s="1"/>
     </row>
@@ -11231,7 +11285,7 @@
         <v>1.45931237591159</v>
       </c>
       <c r="D121" s="12">
-        <v>0.78240753934795104</v>
+        <v>0.76245692349070604</v>
       </c>
       <c r="E121" s="12">
         <v>3.3733094604205101</v>
@@ -11243,10 +11297,10 @@
         <v>-2.2889039419712902</v>
       </c>
       <c r="H121" s="12">
-        <v>19.118245204086499</v>
+        <v>18.9662833166926</v>
       </c>
       <c r="I121" s="12">
-        <v>3.1767585695207501</v>
+        <v>3.1651334114635201</v>
       </c>
       <c r="K121" s="1"/>
     </row>
@@ -11258,7 +11312,7 @@
         <v>16.1802925760467</v>
       </c>
       <c r="D122" s="12">
-        <v>11.9746416696604</v>
+        <v>11.974544160933901</v>
       </c>
       <c r="E122" s="12">
         <v>-5.6614115014834798</v>
@@ -11270,100 +11324,118 @@
         <v>9.49079036829648</v>
       </c>
       <c r="H122" s="12">
-        <v>6.5290642010867197</v>
+        <v>6.3896810174956</v>
       </c>
       <c r="I122" s="12">
-        <v>10.200452758813</v>
+        <v>10.194478189113401</v>
       </c>
       <c r="K122" s="1"/>
     </row>
     <row r="123" spans="2:11">
-      <c r="B123" s="33" t="s">
+      <c r="B123" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C123" s="16">
+      <c r="C123" s="12">
         <v>0.57655280366217798</v>
       </c>
-      <c r="D123" s="16">
-        <v>-8.4861005177705506E-2</v>
-      </c>
-      <c r="E123" s="16">
+      <c r="D123" s="12">
+        <v>-8.1868357050396398E-2</v>
+      </c>
+      <c r="E123" s="12">
         <v>-14.657993796920801</v>
       </c>
-      <c r="F123" s="16">
+      <c r="F123" s="12">
         <v>15.343608282550001</v>
       </c>
-      <c r="G123" s="16">
+      <c r="G123" s="12">
         <v>-1.5204325546550701</v>
       </c>
-      <c r="H123" s="16">
-        <v>4.1923386316592</v>
-      </c>
-      <c r="I123" s="16">
-        <v>-1.34462621765121</v>
+      <c r="H123" s="12">
+        <v>4.1775210369299902</v>
+      </c>
+      <c r="I123" s="12">
+        <v>-1.3444392397132101</v>
       </c>
       <c r="K123" s="1"/>
     </row>
-    <row r="124" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B124" s="29" t="s">
+    <row r="124" spans="2:11">
+      <c r="B124" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C124" s="16">
+        <v>2.1201623244404302</v>
+      </c>
+      <c r="D124" s="16">
+        <v>-3.7559979561316599</v>
+      </c>
+      <c r="E124" s="16">
+        <v>-22.411268647167599</v>
+      </c>
+      <c r="F124" s="16">
+        <v>18.123377294566499</v>
+      </c>
+      <c r="G124" s="16">
+        <v>-1.3542187162241599</v>
+      </c>
+      <c r="H124" s="16">
+        <v>5.6151789259897704</v>
+      </c>
+      <c r="I124" s="16">
+        <v>-2.8613489928644902</v>
+      </c>
+      <c r="K124" s="1"/>
+    </row>
+    <row r="125" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B125" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C124" s="30"/>
-      <c r="D124" s="30"/>
-      <c r="E124" s="30"/>
-      <c r="F124" s="30"/>
-      <c r="G124" s="30"/>
-      <c r="H124" s="30"/>
-      <c r="I124" s="30"/>
-      <c r="K124" s="1"/>
-    </row>
-    <row r="125" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B125" s="35" t="s">
+      <c r="C125" s="30"/>
+      <c r="D125" s="30"/>
+      <c r="E125" s="30"/>
+      <c r="F125" s="30"/>
+      <c r="G125" s="30"/>
+      <c r="H125" s="30"/>
+      <c r="I125" s="30"/>
+      <c r="K125" s="1"/>
+    </row>
+    <row r="126" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B126" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C125" s="35"/>
-      <c r="D125" s="35"/>
-      <c r="E125" s="35"/>
-      <c r="F125" s="35"/>
-      <c r="G125" s="35"/>
-      <c r="H125" s="35"/>
-      <c r="I125" s="35"/>
-      <c r="K125" s="1"/>
-    </row>
-    <row r="126" spans="2:11">
-      <c r="B126" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C126" s="32"/>
-      <c r="D126" s="32"/>
-      <c r="E126" s="32"/>
-      <c r="F126" s="32"/>
-      <c r="G126" s="32"/>
-      <c r="H126" s="32"/>
-      <c r="I126" s="32"/>
+      <c r="C126" s="35"/>
+      <c r="D126" s="35"/>
+      <c r="E126" s="35"/>
+      <c r="F126" s="35"/>
+      <c r="G126" s="35"/>
+      <c r="H126" s="35"/>
+      <c r="I126" s="35"/>
       <c r="K126" s="1"/>
     </row>
     <row r="127" spans="2:11">
       <c r="B127" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C127" s="32"/>
+      <c r="D127" s="32"/>
+      <c r="E127" s="32"/>
+      <c r="F127" s="32"/>
+      <c r="G127" s="32"/>
+      <c r="H127" s="32"/>
+      <c r="I127" s="32"/>
+      <c r="K127" s="1"/>
+    </row>
+    <row r="128" spans="2:11">
+      <c r="B128" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C127" s="30"/>
-      <c r="D127" s="30"/>
-      <c r="E127" s="30"/>
-      <c r="F127" s="30"/>
-      <c r="G127" s="30"/>
-      <c r="H127" s="30"/>
-      <c r="I127" s="30"/>
-      <c r="K127" s="1"/>
-    </row>
-    <row r="132" spans="3:9">
-      <c r="C132" s="17"/>
-      <c r="D132" s="17"/>
-      <c r="E132" s="17"/>
-      <c r="F132" s="17"/>
-      <c r="G132" s="17"/>
-      <c r="H132" s="17"/>
-      <c r="I132" s="17"/>
+      <c r="C128" s="30"/>
+      <c r="D128" s="30"/>
+      <c r="E128" s="30"/>
+      <c r="F128" s="30"/>
+      <c r="G128" s="30"/>
+      <c r="H128" s="30"/>
+      <c r="I128" s="30"/>
+      <c r="K128" s="1"/>
     </row>
     <row r="133" spans="3:9">
       <c r="C133" s="17"/>
@@ -11473,14 +11545,14 @@
       <c r="H144" s="17"/>
       <c r="I144" s="17"/>
     </row>
-    <row r="147" spans="3:9">
-      <c r="C147" s="17"/>
-      <c r="D147" s="17"/>
-      <c r="E147" s="17"/>
-      <c r="F147" s="17"/>
-      <c r="G147" s="17"/>
-      <c r="H147" s="17"/>
-      <c r="I147" s="17"/>
+    <row r="145" spans="3:9">
+      <c r="C145" s="17"/>
+      <c r="D145" s="17"/>
+      <c r="E145" s="17"/>
+      <c r="F145" s="17"/>
+      <c r="G145" s="17"/>
+      <c r="H145" s="17"/>
+      <c r="I145" s="17"/>
     </row>
     <row r="148" spans="3:9">
       <c r="C148" s="17"/>
@@ -11581,10 +11653,19 @@
       <c r="H158" s="17"/>
       <c r="I158" s="17"/>
     </row>
+    <row r="159" spans="3:9">
+      <c r="C159" s="17"/>
+      <c r="D159" s="17"/>
+      <c r="E159" s="17"/>
+      <c r="F159" s="17"/>
+      <c r="G159" s="17"/>
+      <c r="H159" s="17"/>
+      <c r="I159" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B125:I125"/>
+    <mergeCell ref="B126:I126"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>